<commit_message>
feat: search.xlsx 4컬럼 동적 반영 및 ipchal.md 세션 8·9 기록 추가
- load_keyword_presets()를 (컬럼명, 키워드목록) 튜플 리스트로 변경하여 컬럼 수에 관계없이 동적 처리
- 멀티셀렉트를 하드코딩 3개에서 Excel 컬럼 수에 맞게 동적 생성으로 전환
- search.xlsx에 대표님 컬럼 추가 반영 (총 4컬럼: 대표님/1순위/2순위/3순위)
- ipchal.md: 세션 8(사전규격 버그 수정·UI 개선), 세션 9(search.xlsx 동적 구조 전환) 기록 추가

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/search.xlsx
+++ b/search.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hb\OneDrive\바탕 화면\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\82104\g2b_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{54A10C7E-9708-4710-B427-2A6A44C3AB57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{CF6EBE31-120E-4462-827D-356C2A028805}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="85">
   <si>
     <t>1순위</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -278,13 +277,89 @@
   </si>
   <si>
     <t>고령</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일자리</t>
+  </si>
+  <si>
+    <t>퇴직</t>
+  </si>
+  <si>
+    <t>은퇴</t>
+  </si>
+  <si>
+    <t>이직</t>
+  </si>
+  <si>
+    <t>전직</t>
+  </si>
+  <si>
+    <t>구직</t>
+  </si>
+  <si>
+    <t>설계</t>
+  </si>
+  <si>
+    <t>경력</t>
+  </si>
+  <si>
+    <t>장년</t>
+  </si>
+  <si>
+    <t xml:space="preserve">중년 </t>
+  </si>
+  <si>
+    <t>시니어</t>
+  </si>
+  <si>
+    <t>부머</t>
+  </si>
+  <si>
+    <t>노인</t>
+  </si>
+  <si>
+    <t>어르신</t>
+  </si>
+  <si>
+    <t>스마트</t>
+  </si>
+  <si>
+    <t>경로당</t>
+  </si>
+  <si>
+    <t>재취업</t>
+  </si>
+  <si>
+    <t>취업</t>
+  </si>
+  <si>
+    <t>창업</t>
+  </si>
+  <si>
+    <t>멘토링</t>
+  </si>
+  <si>
+    <t>인턴십</t>
+  </si>
+  <si>
+    <t>사회적</t>
+  </si>
+  <si>
+    <t>디지털</t>
+  </si>
+  <si>
+    <t>박람회</t>
+  </si>
+  <si>
+    <t>대표님</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -664,294 +739,369 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8814C0C6-C8EF-4152-BEB7-EF945B5DB968}">
-  <dimension ref="A1:C32"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D32"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="8" max="8" width="18.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="1"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="1"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="1"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="1"/>
       <c r="C18" s="1"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="D18" s="1"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="1"/>
       <c r="C19" s="1"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+      <c r="D19" s="1"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="1"/>
       <c r="C20" s="1"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+      <c r="D20" s="1"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="1"/>
       <c r="C21" s="1"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="D21" s="1"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="1"/>
       <c r="C22" s="1"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+      <c r="D22" s="1"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="1"/>
       <c r="C23" s="1"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+      <c r="D23" s="1"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>82</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="1"/>
       <c r="C24" s="1"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+      <c r="D24" s="1"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="1"/>
       <c r="C25" s="1"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="D25" s="1"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B26" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="1"/>
       <c r="C26" s="1"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+      <c r="D26" s="1"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B27" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="1"/>
       <c r="C27" s="1"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="D27" s="1"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B28" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="1"/>
       <c r="C28" s="1"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
+      <c r="D28" s="1"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="1"/>
       <c r="C29" s="1"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+      <c r="D29" s="1"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="1"/>
       <c r="C30" s="1"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+      <c r="D30" s="1"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B31" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="1"/>
       <c r="C31" s="1"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+      <c r="D31" s="1"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B32" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="1"/>
       <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>